<commit_message>
V2 board and updated source
</commit_message>
<xml_diff>
--- a/PCB/BOM.xlsx
+++ b/PCB/BOM.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_Board1_OXFP_2025-06-25" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_Board1_OXFP_2025-08-18" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="43">
   <si>
     <t>No.</t>
   </si>
@@ -49,7 +49,7 @@
     <t>Test-Point</t>
   </si>
   <si>
-    <t>5V</t>
+    <t>5V,GND</t>
   </si>
   <si>
     <t>Test-Point-0.5mm</t>
@@ -61,19 +61,19 @@
     <t>2</t>
   </si>
   <si>
-    <t>B3F-1000</t>
+    <t>TSC015B07518A02</t>
   </si>
   <si>
     <t>EJECT,POWER</t>
   </si>
   <si>
-    <t>KEY-TH_4P-L6.2-W6.2-P4.50-LS6.5</t>
-  </si>
-  <si>
-    <t>OMRON(欧姆龙)</t>
-  </si>
-  <si>
-    <t>C93157</t>
+    <t>SW-SMD_4P-L4.5-W4.5-P3.00-LS6.8</t>
+  </si>
+  <si>
+    <t>BZCN(博众电气)</t>
+  </si>
+  <si>
+    <t>C2888739</t>
   </si>
   <si>
     <t>LCSC</t>
@@ -115,16 +115,31 @@
     <t>5</t>
   </si>
   <si>
-    <t>ESP32-S3-Zero</t>
-  </si>
-  <si>
-    <t>U1</t>
+    <t>SH1.0-3P</t>
+  </si>
+  <si>
+    <t>RGBO1,RGBO2</t>
+  </si>
+  <si>
+    <t>CONN-SMD_3P-P1.00-L5.0-W5.0</t>
+  </si>
+  <si>
+    <t>C9900019066</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>ESP32-C6-Zero</t>
+  </si>
+  <si>
+    <t>U2</t>
   </si>
   <si>
     <t>COMM-SMD_18P-P2.54-L23.5-W18.0-TL</t>
   </si>
   <si>
-    <t>C9900152785</t>
+    <t>C9900163612</t>
   </si>
 </sst>
 </file>
@@ -501,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -544,7 +559,7 @@
         <v>10</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
         <v>11</v>
@@ -672,7 +687,7 @@
         <v>33</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="s">
         <v>34</v>
@@ -699,8 +714,40 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" t="s">
+        <v>42</v>
+      </c>
+      <c r="J7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>